<commit_message>
Working on the Sample Data to run the baseline Models
</commit_message>
<xml_diff>
--- a/data/YourName.xlsx
+++ b/data/YourName.xlsx
@@ -425,482 +425,482 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>152.4485</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>201.6420000000002</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>200.6059999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>200.6059999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>200.4859999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>200.2459999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>200.2459999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>200.2459999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>201.21</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>201.21</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>201.21</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>201.21</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>201.1235</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>201.1235</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>201.1235</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>201.1235</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>202.3999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>201.5955000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>201.337</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>201.37</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>202.2499999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>202.4745</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>202.2634999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>202.1354999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>204.0054999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>202.7805</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>203.546</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>204.7035</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>205.3485</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>204.2834999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>202.1549999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>202.584</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>203.457</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>252.5584999999998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>252.4249999999998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>252.7019999999997</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>253.2824999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>253.2519999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>253.3079999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>252.9924999999998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>253.0714999999998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>254.3955</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>254.4045</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>254.2855</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>264.5755</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>263.4399999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>256.073</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>267.5745000000003</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>255.1099999999998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>265.6924999999998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>269.2765000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>256.0135000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>255.2044999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>270.9800000000002</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>271.2195000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>255.1285000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>270.8140000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>266.9084999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>255.0355</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>259.1039999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>255.431</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>256.2499999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>258.4515</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>255.4569999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>260.941</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>258.5475</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>255.811</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>253.883</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>253.879</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>255.6545</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>254.0135</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>274.1169999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>298.539</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>286.3885000000002</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>299.0350000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>292.9585000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>297.5045000000002</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>298.86</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>299.0270000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>299.0170000000002</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>241.2609999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>241.2754999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>237.112</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>235.687</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>236.8970000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>228.784</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>224.0165</v>
+        <v>0</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>224.7555</v>
+        <v>0</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>220.298</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>221.514</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>219.969</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>219.8645</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>220.0535000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>176.26</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>178.2665000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>179.8220000000001</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>